<commit_message>
messungsauswertung fertigung der PCB -4h
</commit_message>
<xml_diff>
--- a/Dokumentation/IDVG_BS170_first_jey.xlsx
+++ b/Dokumentation/IDVG_BS170_first_jey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael Watzek\Documents\Diplom_Arbeit\Dokumentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D64D279E-A27A-4E47-BC19-10193C5F0E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6BFBB3-4B70-4344-8C7D-E9AAA3FE4AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{83F75D6B-D159-413A-9677-95128F574C8A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
   <si>
     <t>0x000006</t>
   </si>
@@ -164,10 +164,16 @@
     <t>0.060895</t>
   </si>
   <si>
-    <t>Vg in Volt</t>
-  </si>
-  <si>
-    <t>ID in mA</t>
+    <t>Vadc in Volt</t>
+  </si>
+  <si>
+    <t>Vg</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>ID in uA</t>
   </si>
 </sst>
 </file>
@@ -175,7 +181,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -226,7 +232,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -314,7 +320,681 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
+          <a:endParaRPr lang="de-AT"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>IDVG</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:name>Gleitdurchschnitt</c:name>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="movingAvg"/>
+            <c:period val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Tabelle1!$G$8:$G$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.1000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.3</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.4</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.7</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.2000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.2999999999999998</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Tabelle1!$F$8:$F$33</c:f>
+              <c:numCache>
+                <c:formatCode>0.0000</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>1.4E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9.0000000000000011E-3</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>9.0000000000000011E-3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>9.0000000000000011E-3</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.2E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.8000000000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9.0000000000000011E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.28899999999999998</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.2329999999999999</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>5.907</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>21.088999999999999</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>60.902000000000001</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>60.900000000000006</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>60.894999999999996</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-7934-48F8-9FC2-6D6305A2FAB6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="358278623"/>
+        <c:axId val="358297823"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="358278623"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="3"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-AT"/>
+                  <a:t>VG in mV</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="358297823"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="358297823"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-AT"/>
+                  <a:t>ID in uA</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="1.1755654191973721E-2"/>
+              <c:y val="0.3938734076459009"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="358278623"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
           <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="de-AT"/>
+              <a:t>IDVG</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-AT" baseline="0"/>
+              <a:t> BS170</a:t>
+            </a:r>
+            <a:endParaRPr lang="de-AT"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-AT"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -343,7 +1023,7 @@
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln w="12700">
                 <a:solidFill>
                   <a:schemeClr val="accent1"/>
                 </a:solidFill>
@@ -353,96 +1033,96 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Tabelle1!$F$8:$F$33</c:f>
+              <c:f>Tabelle1!$G$8:$G$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
-                  <c:v>0.46900000000000003</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.156</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.23399999999999999</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.23399999999999999</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.23399999999999999</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.156</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.23399999999999999</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.156</c:v>
+                  <c:v>0.7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.156</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.156</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.23399999999999999</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.313</c:v>
+                  <c:v>1.1000000000000001</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.313</c:v>
+                  <c:v>1.2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.23399999999999999</c:v>
+                  <c:v>1.3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.23399999999999999</c:v>
+                  <c:v>1.4</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.313</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.39100000000000001</c:v>
+                  <c:v>1.6</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.93700000000000006</c:v>
+                  <c:v>1.7</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.9689999999999999</c:v>
+                  <c:v>1.8</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9.5309999999999988</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>40.703000000000003</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>194.92200000000003</c:v>
+                  <c:v>2.1</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>695.93700000000001</c:v>
+                  <c:v>2.2000000000000002</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>2009.7659999999998</c:v>
+                  <c:v>2.2999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>2009.6880000000001</c:v>
+                  <c:v>2.4</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>2009.5309999999999</c:v>
+                  <c:v>2.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Tabelle1!$G$8:$G$33</c:f>
+              <c:f>Tabelle1!$F$8:$F$33</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>1.4E-2</c:v>
@@ -528,7 +1208,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-7934-48F8-9FC2-6D6305A2FAB6}"/>
+              <c16:uniqueId val="{00000001-E4C0-408C-8FF2-0B4732D19A9F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -546,7 +1226,6 @@
       <c:valAx>
         <c:axId val="358278623"/>
         <c:scaling>
-          <c:logBase val="10"/>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -664,8 +1343,8 @@
       <c:valAx>
         <c:axId val="358297823"/>
         <c:scaling>
-          <c:logBase val="10"/>
           <c:orientation val="minMax"/>
+          <c:max val="70"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -879,6 +1558,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1395,20 +2114,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>287944</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>135082</xdr:rowOff>
+      <xdr:colOff>728605</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>107867</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>579120</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>625638</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>124497</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1428,6 +2663,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>587511</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>77804</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>483033</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>12791</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Diagramm 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90B0F4F1-CC11-456D-940D-C75DC59F27F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1782,6 +3055,12 @@
         <v>42</v>
       </c>
       <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1798,13 +3077,12 @@
       <c r="E8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F8">
-        <f>D8*1000</f>
-        <v>0.46900000000000003</v>
-      </c>
-      <c r="G8" s="4">
+      <c r="F8" s="4">
         <f>E8*1000</f>
         <v>1.4E-2</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1820,13 +3098,12 @@
       <c r="E9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F9">
-        <f t="shared" ref="F9:F33" si="0">D9*1000</f>
-        <v>0.156</v>
-      </c>
-      <c r="G9" s="4">
-        <f>E9*1000</f>
+      <c r="F9" s="4">
+        <f t="shared" ref="F9:F33" si="0">E9*1000</f>
         <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G9">
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1842,13 +3119,12 @@
       <c r="E10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="4">
         <f t="shared" si="0"/>
-        <v>0.23399999999999999</v>
-      </c>
-      <c r="G10" s="4">
-        <f>E10*1000</f>
         <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G10">
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1864,13 +3140,12 @@
       <c r="E11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="4">
         <f t="shared" si="0"/>
-        <v>0.23399999999999999</v>
-      </c>
-      <c r="G11" s="4">
-        <f>E11*1000</f>
         <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G11">
+        <v>0.3</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1886,13 +3161,12 @@
       <c r="E12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="4">
         <f t="shared" si="0"/>
-        <v>0.23399999999999999</v>
-      </c>
-      <c r="G12" s="4">
-        <f>E12*1000</f>
         <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G12">
+        <v>0.4</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1908,13 +3182,12 @@
       <c r="E13" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="4">
         <f t="shared" si="0"/>
-        <v>0.156</v>
-      </c>
-      <c r="G13" s="4">
-        <f>E13*1000</f>
         <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G13">
+        <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1930,13 +3203,12 @@
       <c r="E14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="4">
         <f t="shared" si="0"/>
-        <v>0.23399999999999999</v>
-      </c>
-      <c r="G14" s="4">
-        <f>E14*1000</f>
         <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G14">
+        <v>0.6</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1952,13 +3224,12 @@
       <c r="E15" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="4">
         <f t="shared" si="0"/>
-        <v>0.156</v>
-      </c>
-      <c r="G15" s="4">
-        <f>E15*1000</f>
         <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G15">
+        <v>0.7</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1974,13 +3245,12 @@
       <c r="E16" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="4">
         <f t="shared" si="0"/>
-        <v>0.156</v>
-      </c>
-      <c r="G16" s="4">
-        <f>E16*1000</f>
         <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G16">
+        <v>0.8</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -1996,13 +3266,12 @@
       <c r="E17" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="4">
         <f t="shared" si="0"/>
-        <v>0.156</v>
-      </c>
-      <c r="G17" s="4">
-        <f>E17*1000</f>
         <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G17">
+        <v>0.9</v>
       </c>
     </row>
     <row r="18" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2018,13 +3287,12 @@
       <c r="E18" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="4">
         <f t="shared" si="0"/>
-        <v>0.23399999999999999</v>
-      </c>
-      <c r="G18" s="4">
-        <f>E18*1000</f>
         <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2040,13 +3308,12 @@
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="4">
         <f t="shared" si="0"/>
-        <v>0.313</v>
-      </c>
-      <c r="G19" s="4">
-        <f>E19*1000</f>
         <v>9.0000000000000011E-3</v>
+      </c>
+      <c r="G19">
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="20" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2062,13 +3329,12 @@
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="4">
         <f t="shared" si="0"/>
-        <v>0.313</v>
-      </c>
-      <c r="G20" s="4">
-        <f>E20*1000</f>
         <v>9.0000000000000011E-3</v>
+      </c>
+      <c r="G20">
+        <v>1.2</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2084,13 +3350,12 @@
       <c r="E21" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="4">
         <f t="shared" si="0"/>
-        <v>0.23399999999999999</v>
-      </c>
-      <c r="G21" s="4">
-        <f>E21*1000</f>
         <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G21">
+        <v>1.3</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2106,13 +3371,12 @@
       <c r="E22" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="4">
         <f t="shared" si="0"/>
-        <v>0.23399999999999999</v>
-      </c>
-      <c r="G22" s="4">
-        <f>E22*1000</f>
         <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G22">
+        <v>1.4</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2128,13 +3392,12 @@
       <c r="E23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="4">
         <f t="shared" si="0"/>
-        <v>0.313</v>
-      </c>
-      <c r="G23" s="4">
-        <f>E23*1000</f>
         <v>9.0000000000000011E-3</v>
+      </c>
+      <c r="G23">
+        <v>1.5</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2150,13 +3413,12 @@
       <c r="E24" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="4">
         <f t="shared" si="0"/>
-        <v>0.39100000000000001</v>
-      </c>
-      <c r="G24" s="4">
-        <f>E24*1000</f>
         <v>1.2E-2</v>
+      </c>
+      <c r="G24">
+        <v>1.6</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2172,13 +3434,12 @@
       <c r="E25" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="4">
         <f t="shared" si="0"/>
-        <v>0.93700000000000006</v>
-      </c>
-      <c r="G25" s="4">
-        <f>E25*1000</f>
         <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="G25">
+        <v>1.7</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2194,13 +3455,12 @@
       <c r="E26" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="4">
         <f t="shared" si="0"/>
-        <v>2.9689999999999999</v>
-      </c>
-      <c r="G26" s="4">
-        <f>E26*1000</f>
         <v>9.0000000000000011E-2</v>
+      </c>
+      <c r="G26">
+        <v>1.8</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2216,13 +3476,12 @@
       <c r="E27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="4">
         <f t="shared" si="0"/>
-        <v>9.5309999999999988</v>
-      </c>
-      <c r="G27" s="4">
-        <f>E27*1000</f>
         <v>0.28899999999999998</v>
+      </c>
+      <c r="G27">
+        <v>1.9</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2238,13 +3497,12 @@
       <c r="E28" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="4">
         <f t="shared" si="0"/>
-        <v>40.703000000000003</v>
-      </c>
-      <c r="G28" s="4">
-        <f>E28*1000</f>
         <v>1.2329999999999999</v>
+      </c>
+      <c r="G28">
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2260,13 +3518,12 @@
       <c r="E29" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="4">
         <f t="shared" si="0"/>
-        <v>194.92200000000003</v>
-      </c>
-      <c r="G29" s="4">
-        <f>E29*1000</f>
         <v>5.907</v>
+      </c>
+      <c r="G29">
+        <v>2.1</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2282,13 +3539,12 @@
       <c r="E30" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="4">
         <f t="shared" si="0"/>
-        <v>695.93700000000001</v>
-      </c>
-      <c r="G30" s="4">
-        <f>E30*1000</f>
         <v>21.088999999999999</v>
+      </c>
+      <c r="G30">
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2304,13 +3560,12 @@
       <c r="E31" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="4">
         <f t="shared" si="0"/>
-        <v>2009.7659999999998</v>
-      </c>
-      <c r="G31" s="4">
-        <f>E31*1000</f>
         <v>60.902000000000001</v>
+      </c>
+      <c r="G31">
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2326,13 +3581,12 @@
       <c r="E32" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="4">
         <f t="shared" si="0"/>
-        <v>2009.6880000000001</v>
-      </c>
-      <c r="G32" s="4">
-        <f>E32*1000</f>
         <v>60.900000000000006</v>
+      </c>
+      <c r="G32">
+        <v>2.4</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="15" x14ac:dyDescent="0.3">
@@ -2348,13 +3602,12 @@
       <c r="E33" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="4">
         <f t="shared" si="0"/>
-        <v>2009.5309999999999</v>
-      </c>
-      <c r="G33" s="4">
-        <f>E33*1000</f>
         <v>60.894999999999996</v>
+      </c>
+      <c r="G33">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -2364,6 +3617,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010056D9870184CB754DB09140706F8229B0" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8e789435dd70ab2d27d0be8757610b78">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="f243c36f-d931-4ec2-a9e2-70b76878fd0f" xmlns:ns4="7d1486ae-ff17-4b97-a920-c7e7a1dad0d2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b68fef88630c2bb2947542bc2ed9d7d0" ns3:_="" ns4:_="">
     <xsd:import namespace="f243c36f-d931-4ec2-a9e2-70b76878fd0f"/>
@@ -2616,15 +3878,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2634,6 +3887,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C79DAE76-FDB6-4197-8DB3-78E58589D1AB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29A9A745-CDCF-45F8-A6B6-BA46DD308832}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2648,14 +3909,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C79DAE76-FDB6-4197-8DB3-78E58589D1AB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>